<commit_message>
Completed Iteration 3 of Gantt Chart. Added progress report
</commit_message>
<xml_diff>
--- a/Iteration-2/Agile Gantt chart.xlsx
+++ b/Iteration-2/Agile Gantt chart.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E7D27BA-5FF5-40AF-B1E7-43DD179BBD4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063A265A-B824-4D63-AB1B-076B7492FFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29660" windowHeight="18620" tabRatio="415" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="415" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="12" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="41">
   <si>
     <t>Task 3</t>
   </si>
@@ -183,6 +183,18 @@
     <t xml:space="preserve">•  Use Progress to add how much of the project you finished by adding a percentage number. 
 •  Add the day you started your project in the Start Date. 
 •  Finish your calculations by filling in the number of days you need to complete your project in the No. of Days field. </t>
+  </si>
+  <si>
+    <t>Stakeholder Register</t>
+  </si>
+  <si>
+    <t>Euan</t>
+  </si>
+  <si>
+    <t>User Persona</t>
+  </si>
+  <si>
+    <t>Group</t>
   </si>
 </sst>
 </file>
@@ -3290,8 +3302,8 @@
         <v>17</v>
       </c>
       <c r="C6" s="80" cm="1">
-        <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Milestones4352[Start])=0,TODAY(),B11(Milestones4352[Start])),TODAY())</f>
-        <v>46113</v>
+        <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Milestones4352[Start])=0,DATE(2026,2,20),B11(Milestones4352[Start])),DATE(2026,2,20))</f>
+        <v>46073</v>
       </c>
       <c r="D6" s="81"/>
       <c r="E6" s="75"/>
@@ -3300,7 +3312,7 @@
       <c r="H6" s="75"/>
       <c r="I6" s="91" t="str">
         <f ca="1">TEXT(I7,"mmmm")</f>
-        <v>April</v>
+        <v>February</v>
       </c>
       <c r="J6" s="91"/>
       <c r="K6" s="91"/>
@@ -3320,7 +3332,7 @@
       <c r="V6" s="91"/>
       <c r="W6" s="91" t="str">
         <f ca="1">IF(OR(TEXT(W7,"mmmm")=P6,TEXT(W7,"mmmm")=I6),"",TEXT(W7,"mmmm"))</f>
-        <v/>
+        <v>March</v>
       </c>
       <c r="X6" s="91"/>
       <c r="Y6" s="91"/>
@@ -3350,7 +3362,7 @@
       <c r="AQ6" s="91"/>
       <c r="AR6" s="91" t="str">
         <f ca="1">IF(OR(TEXT(AR7,"mmmm")=AK6,TEXT(AR7,"mmmm")=AD6,TEXT(AR7,"mmmm")=W6,TEXT(AR7,"mmmm")=P6),"",TEXT(AR7,"mmmm"))</f>
-        <v>May</v>
+        <v/>
       </c>
       <c r="AS6" s="91"/>
       <c r="AT6" s="91"/>
@@ -3360,7 +3372,7 @@
       <c r="AX6" s="92"/>
       <c r="AY6" s="92" t="str">
         <f ca="1">IF(OR(TEXT(AY7,"mmmm")=AR6,TEXT(AY7,"mmmm")=AK6,TEXT(AY7,"mmmm")=AD6,TEXT(AY7,"mmmm")=W6),"",TEXT(AY7,"mmmm"))</f>
-        <v/>
+        <v>April</v>
       </c>
       <c r="AZ6" s="92"/>
       <c r="BA6" s="92"/>
@@ -3394,227 +3406,227 @@
       <c r="H7" s="83"/>
       <c r="I7" s="98">
         <f ca="1">IFERROR(Project_Start+Scrolling_Increment,TODAY())</f>
-        <v>46114</v>
+        <v>46074</v>
       </c>
       <c r="J7" s="99">
         <f ca="1">I7+1</f>
-        <v>46115</v>
+        <v>46075</v>
       </c>
       <c r="K7" s="99">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46116</v>
+        <v>46076</v>
       </c>
       <c r="L7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46117</v>
+        <v>46077</v>
       </c>
       <c r="M7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46118</v>
+        <v>46078</v>
       </c>
       <c r="N7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46119</v>
+        <v>46079</v>
       </c>
       <c r="O7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46120</v>
+        <v>46080</v>
       </c>
       <c r="P7" s="99">
         <f ca="1">O7+1</f>
-        <v>46121</v>
+        <v>46081</v>
       </c>
       <c r="Q7" s="99">
         <f ca="1">P7+1</f>
-        <v>46122</v>
+        <v>46082</v>
       </c>
       <c r="R7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46123</v>
+        <v>46083</v>
       </c>
       <c r="S7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46124</v>
+        <v>46084</v>
       </c>
       <c r="T7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46125</v>
+        <v>46085</v>
       </c>
       <c r="U7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46126</v>
+        <v>46086</v>
       </c>
       <c r="V7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46127</v>
+        <v>46087</v>
       </c>
       <c r="W7" s="99">
         <f ca="1">V7+1</f>
-        <v>46128</v>
+        <v>46088</v>
       </c>
       <c r="X7" s="99">
         <f ca="1">W7+1</f>
-        <v>46129</v>
+        <v>46089</v>
       </c>
       <c r="Y7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46130</v>
+        <v>46090</v>
       </c>
       <c r="Z7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46131</v>
+        <v>46091</v>
       </c>
       <c r="AA7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46132</v>
+        <v>46092</v>
       </c>
       <c r="AB7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46133</v>
+        <v>46093</v>
       </c>
       <c r="AC7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46134</v>
+        <v>46094</v>
       </c>
       <c r="AD7" s="99">
         <f ca="1">AC7+1</f>
-        <v>46135</v>
+        <v>46095</v>
       </c>
       <c r="AE7" s="99">
         <f ca="1">AD7+1</f>
-        <v>46136</v>
+        <v>46096</v>
       </c>
       <c r="AF7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46137</v>
+        <v>46097</v>
       </c>
       <c r="AG7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46138</v>
+        <v>46098</v>
       </c>
       <c r="AH7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46139</v>
+        <v>46099</v>
       </c>
       <c r="AI7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46140</v>
+        <v>46100</v>
       </c>
       <c r="AJ7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46141</v>
+        <v>46101</v>
       </c>
       <c r="AK7" s="99">
         <f ca="1">AJ7+1</f>
-        <v>46142</v>
+        <v>46102</v>
       </c>
       <c r="AL7" s="99">
         <f ca="1">AK7+1</f>
-        <v>46143</v>
+        <v>46103</v>
       </c>
       <c r="AM7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46144</v>
+        <v>46104</v>
       </c>
       <c r="AN7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46145</v>
+        <v>46105</v>
       </c>
       <c r="AO7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46106</v>
       </c>
       <c r="AP7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46147</v>
+        <v>46107</v>
       </c>
       <c r="AQ7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46148</v>
+        <v>46108</v>
       </c>
       <c r="AR7" s="99">
         <f ca="1">AQ7+1</f>
-        <v>46149</v>
+        <v>46109</v>
       </c>
       <c r="AS7" s="99">
         <f ca="1">AR7+1</f>
-        <v>46150</v>
+        <v>46110</v>
       </c>
       <c r="AT7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46151</v>
+        <v>46111</v>
       </c>
       <c r="AU7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46152</v>
+        <v>46112</v>
       </c>
       <c r="AV7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46153</v>
+        <v>46113</v>
       </c>
       <c r="AW7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46154</v>
+        <v>46114</v>
       </c>
       <c r="AX7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46155</v>
+        <v>46115</v>
       </c>
       <c r="AY7" s="99">
         <f ca="1">AX7+1</f>
-        <v>46156</v>
+        <v>46116</v>
       </c>
       <c r="AZ7" s="99">
         <f ca="1">AY7+1</f>
-        <v>46157</v>
+        <v>46117</v>
       </c>
       <c r="BA7" s="99">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46158</v>
+        <v>46118</v>
       </c>
       <c r="BB7" s="99">
         <f t="shared" ca="1" si="1"/>
-        <v>46159</v>
+        <v>46119</v>
       </c>
       <c r="BC7" s="99">
         <f t="shared" ca="1" si="1"/>
-        <v>46160</v>
+        <v>46120</v>
       </c>
       <c r="BD7" s="99">
         <f t="shared" ca="1" si="1"/>
-        <v>46161</v>
+        <v>46121</v>
       </c>
       <c r="BE7" s="100">
         <f t="shared" ca="1" si="1"/>
-        <v>46162</v>
+        <v>46122</v>
       </c>
       <c r="BF7" s="99">
         <f ca="1">BE7+1</f>
-        <v>46163</v>
+        <v>46123</v>
       </c>
       <c r="BG7" s="99">
         <f ca="1">BF7+1</f>
-        <v>46164</v>
+        <v>46124</v>
       </c>
       <c r="BH7" s="99">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46165</v>
+        <v>46125</v>
       </c>
       <c r="BI7" s="99">
         <f t="shared" ca="1" si="2"/>
-        <v>46166</v>
+        <v>46126</v>
       </c>
       <c r="BJ7" s="99">
         <f t="shared" ca="1" si="2"/>
-        <v>46167</v>
+        <v>46127</v>
       </c>
       <c r="BK7" s="99">
         <f t="shared" ca="1" si="2"/>
-        <v>46168</v>
+        <v>46128</v>
       </c>
       <c r="BL7" s="100">
         <f t="shared" ca="1" si="2"/>
-        <v>46169</v>
+        <v>46129</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -3706,23 +3718,23 @@
       <c r="H9" s="88"/>
       <c r="I9" s="106" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="J9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>S</v>
       </c>
       <c r="K9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="L9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="M9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>W</v>
       </c>
       <c r="N9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3730,27 +3742,27 @@
       </c>
       <c r="O9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>F</v>
       </c>
       <c r="P9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="Q9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>S</v>
       </c>
       <c r="R9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="S9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="T9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>W</v>
       </c>
       <c r="U9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3758,27 +3770,27 @@
       </c>
       <c r="V9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>F</v>
       </c>
       <c r="W9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="X9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>S</v>
       </c>
       <c r="Y9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="Z9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="AA9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>W</v>
       </c>
       <c r="AB9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3786,27 +3798,27 @@
       </c>
       <c r="AC9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>F</v>
       </c>
       <c r="AD9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="AE9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>S</v>
       </c>
       <c r="AF9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="AG9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="AH9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>W</v>
       </c>
       <c r="AI9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3814,27 +3826,27 @@
       </c>
       <c r="AJ9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>F</v>
       </c>
       <c r="AK9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="AL9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>S</v>
       </c>
       <c r="AM9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="AN9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="AO9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>W</v>
       </c>
       <c r="AP9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3842,27 +3854,27 @@
       </c>
       <c r="AQ9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>F</v>
       </c>
       <c r="AR9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="AS9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>S</v>
       </c>
       <c r="AT9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="AU9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="AV9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>W</v>
       </c>
       <c r="AW9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3870,27 +3882,27 @@
       </c>
       <c r="AX9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>F</v>
       </c>
       <c r="AY9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="AZ9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>S</v>
       </c>
       <c r="BA9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="BB9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="BC9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>W</v>
       </c>
       <c r="BD9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3898,27 +3910,27 @@
       </c>
       <c r="BE9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>F</v>
       </c>
       <c r="BF9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>S</v>
       </c>
       <c r="BG9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>S</v>
       </c>
       <c r="BH9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>M</v>
       </c>
       <c r="BI9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>T</v>
       </c>
       <c r="BJ9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>W</v>
       </c>
       <c r="BK9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -3926,7 +3938,7 @@
       </c>
       <c r="BL9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>F</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -4233,32 +4245,32 @@
     <row r="12" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10"/>
       <c r="B12" s="63" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="C12" s="59" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D12" s="59" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="E12" s="60">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F12" s="61">
-        <f ca="1">TODAY()</f>
-        <v>46113</v>
+        <f>DATE(2026,2,20)</f>
+        <v>46073</v>
       </c>
       <c r="G12" s="62">
         <v>3</v>
       </c>
       <c r="H12" s="59"/>
-      <c r="I12" s="26">
+      <c r="I12" s="26" t="str">
         <f ca="1">IF(AND($C12="Goal",I$7&gt;=$F12,I$7&lt;=$F12+$G12-1),2,IF(AND($C12="Milestone",I$7&gt;=$F12,I$7&lt;=$F12+$G12-1),1,""))</f>
-        <v>2</v>
-      </c>
-      <c r="J12" s="26">
-        <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v/>
+      </c>
+      <c r="J12" s="26" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v/>
       </c>
       <c r="K12" s="26" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -4480,19 +4492,23 @@
     <row r="13" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10"/>
       <c r="B13" s="63" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C13" s="59" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="59"/>
-      <c r="E13" s="60"/>
+        <v>14</v>
+      </c>
+      <c r="D13" s="59" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="60">
+        <v>1</v>
+      </c>
       <c r="F13" s="61">
-        <f ca="1">TODAY()+5</f>
-        <v>46118</v>
+        <f>DATE(2026,3,4)</f>
+        <v>46085</v>
       </c>
       <c r="G13" s="62">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H13" s="59"/>
       <c r="I13" s="26" t="str">
@@ -4511,9 +4527,9 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="M13" s="26">
-        <f t="shared" ca="1" si="4"/>
-        <v>1</v>
+      <c r="M13" s="26" t="str">
+        <f t="shared" ca="1" si="4"/>
+        <v/>
       </c>
       <c r="N13" s="26" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -4733,8 +4749,8 @@
         <v>0.5</v>
       </c>
       <c r="F14" s="61">
-        <f ca="1">F12-3</f>
-        <v>46110</v>
+        <f>F12-3</f>
+        <v>46070</v>
       </c>
       <c r="G14" s="62">
         <v>10</v>
@@ -4976,8 +4992,8 @@
       <c r="D15" s="59"/>
       <c r="E15" s="60"/>
       <c r="F15" s="61">
-        <f ca="1">F12+20</f>
-        <v>46133</v>
+        <f>F12+20</f>
+        <v>46093</v>
       </c>
       <c r="G15" s="62">
         <v>1</v>
@@ -5221,8 +5237,8 @@
         <v>0.1</v>
       </c>
       <c r="F16" s="61">
-        <f ca="1">F12+6</f>
-        <v>46119</v>
+        <f>F12+6</f>
+        <v>46079</v>
       </c>
       <c r="G16" s="62">
         <v>6</v>
@@ -5702,8 +5718,8 @@
         <v>0.6</v>
       </c>
       <c r="F18" s="61">
-        <f ca="1">F12+6</f>
-        <v>46119</v>
+        <f>F12+6</f>
+        <v>46079</v>
       </c>
       <c r="G18" s="62">
         <v>13</v>
@@ -5947,8 +5963,8 @@
         <v>0.5</v>
       </c>
       <c r="F19" s="61">
-        <f ca="1">F18+2</f>
-        <v>46121</v>
+        <f>F18+2</f>
+        <v>46081</v>
       </c>
       <c r="G19" s="62">
         <v>9</v>
@@ -6192,8 +6208,8 @@
         <v>0.33</v>
       </c>
       <c r="F20" s="61">
-        <f ca="1">F19+5</f>
-        <v>46126</v>
+        <f>F19+5</f>
+        <v>46086</v>
       </c>
       <c r="G20" s="62">
         <v>11</v>
@@ -6435,8 +6451,8 @@
       <c r="D21" s="59"/>
       <c r="E21" s="60"/>
       <c r="F21" s="61">
-        <f ca="1">F20+2</f>
-        <v>46128</v>
+        <f>F20+2</f>
+        <v>46088</v>
       </c>
       <c r="G21" s="62">
         <v>1</v>
@@ -6676,8 +6692,8 @@
       <c r="D22" s="59"/>
       <c r="E22" s="60"/>
       <c r="F22" s="61">
-        <f ca="1">F21+1</f>
-        <v>46129</v>
+        <f>F21+1</f>
+        <v>46089</v>
       </c>
       <c r="G22" s="62">
         <v>24</v>
@@ -7155,8 +7171,8 @@
       <c r="D24" s="59"/>
       <c r="E24" s="60"/>
       <c r="F24" s="61">
-        <f ca="1">F12+15</f>
-        <v>46128</v>
+        <f>F12+15</f>
+        <v>46088</v>
       </c>
       <c r="G24" s="62">
         <v>4</v>
@@ -7398,8 +7414,8 @@
       <c r="D25" s="59"/>
       <c r="E25" s="60"/>
       <c r="F25" s="61">
-        <f ca="1">F24+3</f>
-        <v>46131</v>
+        <f>F24+3</f>
+        <v>46091</v>
       </c>
       <c r="G25" s="62">
         <v>14</v>
@@ -7641,8 +7657,8 @@
       <c r="D26" s="59"/>
       <c r="E26" s="60"/>
       <c r="F26" s="61">
-        <f ca="1">F25+15</f>
-        <v>46146</v>
+        <f>F25+15</f>
+        <v>46106</v>
       </c>
       <c r="G26" s="62">
         <v>6</v>
@@ -7884,8 +7900,8 @@
       <c r="D27" s="59"/>
       <c r="E27" s="60"/>
       <c r="F27" s="61">
-        <f ca="1">F21+22</f>
-        <v>46150</v>
+        <f>F21+22</f>
+        <v>46110</v>
       </c>
       <c r="G27" s="62">
         <v>3</v>
@@ -8127,8 +8143,8 @@
       <c r="D28" s="59"/>
       <c r="E28" s="60"/>
       <c r="F28" s="61">
-        <f ca="1">F16</f>
-        <v>46119</v>
+        <f>F16</f>
+        <v>46079</v>
       </c>
       <c r="G28" s="62">
         <v>19</v>
@@ -8604,8 +8620,8 @@
       <c r="D30" s="59"/>
       <c r="E30" s="60"/>
       <c r="F30" s="61">
-        <f ca="1">F27+3</f>
-        <v>46153</v>
+        <f>F27+3</f>
+        <v>46113</v>
       </c>
       <c r="G30" s="62">
         <v>15</v>
@@ -8845,8 +8861,8 @@
       <c r="D31" s="59"/>
       <c r="E31" s="60"/>
       <c r="F31" s="61">
-        <f ca="1">F30+14</f>
-        <v>46167</v>
+        <f>F30+14</f>
+        <v>46127</v>
       </c>
       <c r="G31" s="62">
         <v>5</v>
@@ -9088,8 +9104,8 @@
       <c r="D32" s="59"/>
       <c r="E32" s="60"/>
       <c r="F32" s="61">
-        <f ca="1">F31+42</f>
-        <v>46209</v>
+        <f>F31+42</f>
+        <v>46169</v>
       </c>
       <c r="G32" s="62">
         <v>1</v>
@@ -10618,7 +10634,7 @@
       </c>
       <c r="C6" s="34" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Milestones435[Start])=0,TODAY(),B11(Milestones435[Start])),TODAY())</f>
-        <v>46113</v>
+        <v>46140</v>
       </c>
       <c r="D6" s="53"/>
       <c r="E6" s="32"/>
@@ -10637,7 +10653,7 @@
       <c r="O6" s="94"/>
       <c r="P6" s="94" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>May</v>
       </c>
       <c r="Q6" s="94"/>
       <c r="R6" s="94"/>
@@ -10677,7 +10693,7 @@
       <c r="AQ6" s="94"/>
       <c r="AR6" s="94" t="str">
         <f ca="1">IF(OR(TEXT(AR7,"mmmm")=AK6,TEXT(AR7,"mmmm")=AD6,TEXT(AR7,"mmmm")=W6,TEXT(AR7,"mmmm")=P6),"",TEXT(AR7,"mmmm"))</f>
-        <v>May</v>
+        <v>June</v>
       </c>
       <c r="AS6" s="94"/>
       <c r="AT6" s="94"/>
@@ -10722,227 +10738,227 @@
       <c r="H7" s="29"/>
       <c r="I7" s="96">
         <f ca="1">IFERROR(Project_Start+Scrolling_Increment,TODAY())</f>
-        <v>46114</v>
+        <v>46141</v>
       </c>
       <c r="J7" s="17">
         <f ca="1">I7+1</f>
-        <v>46115</v>
+        <v>46142</v>
       </c>
       <c r="K7" s="17">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46116</v>
+        <v>46143</v>
       </c>
       <c r="L7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46117</v>
+        <v>46144</v>
       </c>
       <c r="M7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46118</v>
+        <v>46145</v>
       </c>
       <c r="N7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="O7" s="64">
         <f t="shared" ca="1" si="0"/>
-        <v>46120</v>
+        <v>46147</v>
       </c>
       <c r="P7" s="17">
         <f ca="1">O7+1</f>
-        <v>46121</v>
+        <v>46148</v>
       </c>
       <c r="Q7" s="17">
         <f ca="1">P7+1</f>
-        <v>46122</v>
+        <v>46149</v>
       </c>
       <c r="R7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46123</v>
+        <v>46150</v>
       </c>
       <c r="S7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46124</v>
+        <v>46151</v>
       </c>
       <c r="T7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46125</v>
+        <v>46152</v>
       </c>
       <c r="U7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46126</v>
+        <v>46153</v>
       </c>
       <c r="V7" s="64">
         <f t="shared" ca="1" si="0"/>
-        <v>46127</v>
+        <v>46154</v>
       </c>
       <c r="W7" s="17">
         <f ca="1">V7+1</f>
-        <v>46128</v>
+        <v>46155</v>
       </c>
       <c r="X7" s="17">
         <f ca="1">W7+1</f>
-        <v>46129</v>
+        <v>46156</v>
       </c>
       <c r="Y7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46130</v>
+        <v>46157</v>
       </c>
       <c r="Z7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46131</v>
+        <v>46158</v>
       </c>
       <c r="AA7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46132</v>
+        <v>46159</v>
       </c>
       <c r="AB7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46133</v>
+        <v>46160</v>
       </c>
       <c r="AC7" s="64">
         <f t="shared" ca="1" si="0"/>
-        <v>46134</v>
+        <v>46161</v>
       </c>
       <c r="AD7" s="17">
         <f ca="1">AC7+1</f>
-        <v>46135</v>
+        <v>46162</v>
       </c>
       <c r="AE7" s="17">
         <f ca="1">AD7+1</f>
-        <v>46136</v>
+        <v>46163</v>
       </c>
       <c r="AF7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46137</v>
+        <v>46164</v>
       </c>
       <c r="AG7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46138</v>
+        <v>46165</v>
       </c>
       <c r="AH7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46139</v>
+        <v>46166</v>
       </c>
       <c r="AI7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46140</v>
+        <v>46167</v>
       </c>
       <c r="AJ7" s="64">
         <f t="shared" ca="1" si="0"/>
-        <v>46141</v>
+        <v>46168</v>
       </c>
       <c r="AK7" s="17">
         <f ca="1">AJ7+1</f>
-        <v>46142</v>
+        <v>46169</v>
       </c>
       <c r="AL7" s="17">
         <f ca="1">AK7+1</f>
-        <v>46143</v>
+        <v>46170</v>
       </c>
       <c r="AM7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46144</v>
+        <v>46171</v>
       </c>
       <c r="AN7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46145</v>
+        <v>46172</v>
       </c>
       <c r="AO7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46146</v>
+        <v>46173</v>
       </c>
       <c r="AP7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46147</v>
+        <v>46174</v>
       </c>
       <c r="AQ7" s="64">
         <f t="shared" ca="1" si="0"/>
-        <v>46148</v>
+        <v>46175</v>
       </c>
       <c r="AR7" s="17">
         <f ca="1">AQ7+1</f>
-        <v>46149</v>
+        <v>46176</v>
       </c>
       <c r="AS7" s="17">
         <f ca="1">AR7+1</f>
-        <v>46150</v>
+        <v>46177</v>
       </c>
       <c r="AT7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46151</v>
+        <v>46178</v>
       </c>
       <c r="AU7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46152</v>
+        <v>46179</v>
       </c>
       <c r="AV7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46153</v>
+        <v>46180</v>
       </c>
       <c r="AW7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>46154</v>
+        <v>46181</v>
       </c>
       <c r="AX7" s="64">
         <f t="shared" ca="1" si="0"/>
-        <v>46155</v>
+        <v>46182</v>
       </c>
       <c r="AY7" s="17">
         <f ca="1">AX7+1</f>
-        <v>46156</v>
+        <v>46183</v>
       </c>
       <c r="AZ7" s="17">
         <f ca="1">AY7+1</f>
-        <v>46157</v>
+        <v>46184</v>
       </c>
       <c r="BA7" s="17">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46158</v>
+        <v>46185</v>
       </c>
       <c r="BB7" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>46159</v>
+        <v>46186</v>
       </c>
       <c r="BC7" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>46160</v>
+        <v>46187</v>
       </c>
       <c r="BD7" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>46161</v>
+        <v>46188</v>
       </c>
       <c r="BE7" s="64">
         <f t="shared" ca="1" si="1"/>
-        <v>46162</v>
+        <v>46189</v>
       </c>
       <c r="BF7" s="17">
         <f ca="1">BE7+1</f>
-        <v>46163</v>
+        <v>46190</v>
       </c>
       <c r="BG7" s="17">
         <f ca="1">BF7+1</f>
-        <v>46164</v>
+        <v>46191</v>
       </c>
       <c r="BH7" s="17">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46165</v>
+        <v>46192</v>
       </c>
       <c r="BI7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>46166</v>
+        <v>46193</v>
       </c>
       <c r="BJ7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>46167</v>
+        <v>46194</v>
       </c>
       <c r="BK7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>46168</v>
+        <v>46195</v>
       </c>
       <c r="BL7" s="18">
         <f t="shared" ca="1" si="2"/>
-        <v>46169</v>
+        <v>46196</v>
       </c>
       <c r="BM7" s="32"/>
     </row>
@@ -11036,15 +11052,15 @@
       <c r="H9" s="48"/>
       <c r="I9" s="37" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="J9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="K9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="L9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11052,27 +11068,27 @@
       </c>
       <c r="M9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="N9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="O9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="P9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="Q9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="R9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="S9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11080,27 +11096,27 @@
       </c>
       <c r="T9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="U9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="V9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="W9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="X9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="Y9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="Z9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11108,27 +11124,27 @@
       </c>
       <c r="AA9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="AB9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AC9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="AD9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="AE9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AF9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="AG9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11136,27 +11152,27 @@
       </c>
       <c r="AH9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="AI9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AJ9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="AK9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="AL9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AM9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="AN9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11164,27 +11180,27 @@
       </c>
       <c r="AO9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="AP9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AQ9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="AR9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="AS9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AT9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="AU9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11192,27 +11208,27 @@
       </c>
       <c r="AV9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="AW9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AX9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="AY9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="AZ9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="BA9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="BB9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11220,27 +11236,27 @@
       </c>
       <c r="BC9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="BD9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="BE9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="BF9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="BG9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="BH9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="BI9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -11248,15 +11264,15 @@
       </c>
       <c r="BJ9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="BK9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="BL9" s="37" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="BM9" s="32"/>
     </row>
@@ -11580,7 +11596,7 @@
       </c>
       <c r="F12" s="23">
         <f ca="1">TODAY()</f>
-        <v>46113</v>
+        <v>46140</v>
       </c>
       <c r="G12" s="24">
         <v>3</v>
@@ -11824,7 +11840,7 @@
       <c r="E13" s="22"/>
       <c r="F13" s="23">
         <f ca="1">TODAY()+5</f>
-        <v>46118</v>
+        <v>46145</v>
       </c>
       <c r="G13" s="24">
         <v>1</v>
@@ -12070,7 +12086,7 @@
       </c>
       <c r="F14" s="23">
         <f ca="1">F12-3</f>
-        <v>46110</v>
+        <v>46137</v>
       </c>
       <c r="G14" s="24">
         <v>10</v>
@@ -12314,7 +12330,7 @@
       <c r="E15" s="22"/>
       <c r="F15" s="23">
         <f ca="1">F12+20</f>
-        <v>46133</v>
+        <v>46160</v>
       </c>
       <c r="G15" s="24">
         <v>1</v>
@@ -12560,7 +12576,7 @@
       </c>
       <c r="F16" s="23">
         <f ca="1">F12+6</f>
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="G16" s="24">
         <v>6</v>
@@ -13043,7 +13059,7 @@
       </c>
       <c r="F18" s="23">
         <f ca="1">F12+6</f>
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="G18" s="24">
         <v>13</v>
@@ -13289,7 +13305,7 @@
       </c>
       <c r="F19" s="23">
         <f ca="1">F18+2</f>
-        <v>46121</v>
+        <v>46148</v>
       </c>
       <c r="G19" s="24">
         <v>9</v>
@@ -13535,7 +13551,7 @@
       </c>
       <c r="F20" s="23">
         <f ca="1">F19+5</f>
-        <v>46126</v>
+        <v>46153</v>
       </c>
       <c r="G20" s="24">
         <v>11</v>
@@ -13779,7 +13795,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="23">
         <f ca="1">F20+2</f>
-        <v>46128</v>
+        <v>46155</v>
       </c>
       <c r="G21" s="24">
         <v>1</v>
@@ -14021,7 +14037,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="23">
         <f ca="1">F21+1</f>
-        <v>46129</v>
+        <v>46156</v>
       </c>
       <c r="G22" s="24">
         <v>24</v>
@@ -14502,7 +14518,7 @@
       <c r="E24" s="22"/>
       <c r="F24" s="23">
         <f ca="1">F12+15</f>
-        <v>46128</v>
+        <v>46155</v>
       </c>
       <c r="G24" s="24">
         <v>4</v>
@@ -14746,7 +14762,7 @@
       <c r="E25" s="22"/>
       <c r="F25" s="23">
         <f ca="1">F24+3</f>
-        <v>46131</v>
+        <v>46158</v>
       </c>
       <c r="G25" s="24">
         <v>14</v>
@@ -14990,7 +15006,7 @@
       <c r="E26" s="22"/>
       <c r="F26" s="23">
         <f ca="1">F25+15</f>
-        <v>46146</v>
+        <v>46173</v>
       </c>
       <c r="G26" s="24">
         <v>6</v>
@@ -15234,7 +15250,7 @@
       <c r="E27" s="22"/>
       <c r="F27" s="23">
         <f ca="1">F21+22</f>
-        <v>46150</v>
+        <v>46177</v>
       </c>
       <c r="G27" s="24">
         <v>3</v>
@@ -15478,7 +15494,7 @@
       <c r="E28" s="22"/>
       <c r="F28" s="23">
         <f ca="1">F16</f>
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="G28" s="24">
         <v>19</v>
@@ -15957,7 +15973,7 @@
       <c r="E30" s="22"/>
       <c r="F30" s="23">
         <f ca="1">F27+3</f>
-        <v>46153</v>
+        <v>46180</v>
       </c>
       <c r="G30" s="24">
         <v>15</v>
@@ -16199,7 +16215,7 @@
       <c r="E31" s="22"/>
       <c r="F31" s="23">
         <f ca="1">F30+14</f>
-        <v>46167</v>
+        <v>46194</v>
       </c>
       <c r="G31" s="24">
         <v>5</v>
@@ -16443,7 +16459,7 @@
       <c r="E32" s="22"/>
       <c r="F32" s="23">
         <f ca="1">F31+42</f>
-        <v>46209</v>
+        <v>46236</v>
       </c>
       <c r="G32" s="24">
         <v>1</v>
@@ -17829,7 +17845,7 @@
       </c>
       <c r="C6" s="80" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Milestones43524[Start])=0,TODAY(),B11(Milestones43524[Start])),TODAY())</f>
-        <v>46113</v>
+        <v>46140</v>
       </c>
       <c r="D6" s="81"/>
       <c r="E6" s="75"/>
@@ -17838,7 +17854,7 @@
       <c r="H6" s="75"/>
       <c r="I6" s="91" t="str">
         <f ca="1">TEXT(I7,"mmmm")</f>
-        <v>April</v>
+        <v>May</v>
       </c>
       <c r="J6" s="91"/>
       <c r="K6" s="91"/>
@@ -17878,7 +17894,7 @@
       <c r="AJ6" s="91"/>
       <c r="AK6" s="91" t="str">
         <f ca="1">IF(OR(TEXT(AK7,"mmmm")=AD6,TEXT(AK7,"mmmm")=W6,TEXT(AK7,"mmmm")=P6,TEXT(AK7,"mmmm")=I6),"",TEXT(AK7,"mmmm"))</f>
-        <v>May</v>
+        <v/>
       </c>
       <c r="AL6" s="91"/>
       <c r="AM6" s="91"/>
@@ -17888,7 +17904,7 @@
       <c r="AQ6" s="91"/>
       <c r="AR6" s="91" t="str">
         <f ca="1">IF(OR(TEXT(AR7,"mmmm")=AK6,TEXT(AR7,"mmmm")=AD6,TEXT(AR7,"mmmm")=W6,TEXT(AR7,"mmmm")=P6),"",TEXT(AR7,"mmmm"))</f>
-        <v/>
+        <v>June</v>
       </c>
       <c r="AS6" s="91"/>
       <c r="AT6" s="91"/>
@@ -17932,227 +17948,227 @@
       <c r="H7" s="83"/>
       <c r="I7" s="98">
         <f ca="1">IFERROR(Project_Start+Scrolling_Increment,TODAY())</f>
-        <v>46118</v>
+        <v>46145</v>
       </c>
       <c r="J7" s="99">
         <f ca="1">I7+1</f>
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="K7" s="99">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46120</v>
+        <v>46147</v>
       </c>
       <c r="L7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46121</v>
+        <v>46148</v>
       </c>
       <c r="M7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46122</v>
+        <v>46149</v>
       </c>
       <c r="N7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46123</v>
+        <v>46150</v>
       </c>
       <c r="O7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46124</v>
+        <v>46151</v>
       </c>
       <c r="P7" s="99">
         <f ca="1">O7+1</f>
-        <v>46125</v>
+        <v>46152</v>
       </c>
       <c r="Q7" s="99">
         <f ca="1">P7+1</f>
-        <v>46126</v>
+        <v>46153</v>
       </c>
       <c r="R7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46127</v>
+        <v>46154</v>
       </c>
       <c r="S7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46128</v>
+        <v>46155</v>
       </c>
       <c r="T7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46129</v>
+        <v>46156</v>
       </c>
       <c r="U7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46130</v>
+        <v>46157</v>
       </c>
       <c r="V7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46131</v>
+        <v>46158</v>
       </c>
       <c r="W7" s="99">
         <f ca="1">V7+1</f>
-        <v>46132</v>
+        <v>46159</v>
       </c>
       <c r="X7" s="99">
         <f ca="1">W7+1</f>
-        <v>46133</v>
+        <v>46160</v>
       </c>
       <c r="Y7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46134</v>
+        <v>46161</v>
       </c>
       <c r="Z7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46135</v>
+        <v>46162</v>
       </c>
       <c r="AA7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46136</v>
+        <v>46163</v>
       </c>
       <c r="AB7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46137</v>
+        <v>46164</v>
       </c>
       <c r="AC7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46138</v>
+        <v>46165</v>
       </c>
       <c r="AD7" s="99">
         <f ca="1">AC7+1</f>
-        <v>46139</v>
+        <v>46166</v>
       </c>
       <c r="AE7" s="99">
         <f ca="1">AD7+1</f>
-        <v>46140</v>
+        <v>46167</v>
       </c>
       <c r="AF7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46141</v>
+        <v>46168</v>
       </c>
       <c r="AG7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46142</v>
+        <v>46169</v>
       </c>
       <c r="AH7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46143</v>
+        <v>46170</v>
       </c>
       <c r="AI7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46144</v>
+        <v>46171</v>
       </c>
       <c r="AJ7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46145</v>
+        <v>46172</v>
       </c>
       <c r="AK7" s="99">
         <f ca="1">AJ7+1</f>
-        <v>46146</v>
+        <v>46173</v>
       </c>
       <c r="AL7" s="99">
         <f ca="1">AK7+1</f>
-        <v>46147</v>
+        <v>46174</v>
       </c>
       <c r="AM7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46148</v>
+        <v>46175</v>
       </c>
       <c r="AN7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46149</v>
+        <v>46176</v>
       </c>
       <c r="AO7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46150</v>
+        <v>46177</v>
       </c>
       <c r="AP7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46151</v>
+        <v>46178</v>
       </c>
       <c r="AQ7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46152</v>
+        <v>46179</v>
       </c>
       <c r="AR7" s="99">
         <f ca="1">AQ7+1</f>
-        <v>46153</v>
+        <v>46180</v>
       </c>
       <c r="AS7" s="99">
         <f ca="1">AR7+1</f>
-        <v>46154</v>
+        <v>46181</v>
       </c>
       <c r="AT7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46155</v>
+        <v>46182</v>
       </c>
       <c r="AU7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46156</v>
+        <v>46183</v>
       </c>
       <c r="AV7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46157</v>
+        <v>46184</v>
       </c>
       <c r="AW7" s="99">
         <f t="shared" ca="1" si="0"/>
-        <v>46158</v>
+        <v>46185</v>
       </c>
       <c r="AX7" s="100">
         <f t="shared" ca="1" si="0"/>
-        <v>46159</v>
+        <v>46186</v>
       </c>
       <c r="AY7" s="99">
         <f ca="1">AX7+1</f>
-        <v>46160</v>
+        <v>46187</v>
       </c>
       <c r="AZ7" s="99">
         <f ca="1">AY7+1</f>
-        <v>46161</v>
+        <v>46188</v>
       </c>
       <c r="BA7" s="99">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46162</v>
+        <v>46189</v>
       </c>
       <c r="BB7" s="99">
         <f t="shared" ca="1" si="1"/>
-        <v>46163</v>
+        <v>46190</v>
       </c>
       <c r="BC7" s="99">
         <f t="shared" ca="1" si="1"/>
-        <v>46164</v>
+        <v>46191</v>
       </c>
       <c r="BD7" s="99">
         <f t="shared" ca="1" si="1"/>
-        <v>46165</v>
+        <v>46192</v>
       </c>
       <c r="BE7" s="100">
         <f t="shared" ca="1" si="1"/>
-        <v>46166</v>
+        <v>46193</v>
       </c>
       <c r="BF7" s="99">
         <f ca="1">BE7+1</f>
-        <v>46167</v>
+        <v>46194</v>
       </c>
       <c r="BG7" s="99">
         <f ca="1">BF7+1</f>
-        <v>46168</v>
+        <v>46195</v>
       </c>
       <c r="BH7" s="99">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46169</v>
+        <v>46196</v>
       </c>
       <c r="BI7" s="99">
         <f t="shared" ca="1" si="2"/>
-        <v>46170</v>
+        <v>46197</v>
       </c>
       <c r="BJ7" s="99">
         <f t="shared" ca="1" si="2"/>
-        <v>46171</v>
+        <v>46198</v>
       </c>
       <c r="BK7" s="99">
         <f t="shared" ca="1" si="2"/>
-        <v>46172</v>
+        <v>46199</v>
       </c>
       <c r="BL7" s="100">
         <f t="shared" ca="1" si="2"/>
-        <v>46173</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -18244,27 +18260,27 @@
       <c r="H9" s="88"/>
       <c r="I9" s="106" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="J9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="K9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="L9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="M9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="N9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="O9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18272,27 +18288,27 @@
       </c>
       <c r="P9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="Q9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="R9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="S9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="T9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="U9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="V9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18300,27 +18316,27 @@
       </c>
       <c r="W9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="X9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="Y9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="Z9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="AA9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AB9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="AC9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18328,27 +18344,27 @@
       </c>
       <c r="AD9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="AE9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AF9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="AG9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="AH9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AI9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="AJ9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18356,27 +18372,27 @@
       </c>
       <c r="AK9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="AL9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AM9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="AN9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="AO9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AP9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="AQ9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18384,27 +18400,27 @@
       </c>
       <c r="AR9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="AS9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="AT9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="AU9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="AV9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AW9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="AX9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18412,27 +18428,27 @@
       </c>
       <c r="AY9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="AZ9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="BA9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="BB9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="BC9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="BD9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="BE9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18440,27 +18456,27 @@
       </c>
       <c r="BF9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>M</v>
+        <v>S</v>
       </c>
       <c r="BG9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>M</v>
       </c>
       <c r="BH9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>W</v>
+        <v>T</v>
       </c>
       <c r="BI9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>T</v>
+        <v>W</v>
       </c>
       <c r="BJ9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="BK9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>S</v>
+        <v>F</v>
       </c>
       <c r="BL9" s="106" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -18784,7 +18800,7 @@
       </c>
       <c r="F12" s="61">
         <f ca="1">TODAY()</f>
-        <v>46113</v>
+        <v>46140</v>
       </c>
       <c r="G12" s="62">
         <v>3</v>
@@ -19027,7 +19043,7 @@
       <c r="E13" s="60"/>
       <c r="F13" s="61">
         <f ca="1">TODAY()+5</f>
-        <v>46118</v>
+        <v>46145</v>
       </c>
       <c r="G13" s="62">
         <v>1</v>
@@ -19272,7 +19288,7 @@
       </c>
       <c r="F14" s="61">
         <f ca="1">F12-3</f>
-        <v>46110</v>
+        <v>46137</v>
       </c>
       <c r="G14" s="62">
         <v>10</v>
@@ -19515,7 +19531,7 @@
       <c r="E15" s="60"/>
       <c r="F15" s="61">
         <f ca="1">F12+20</f>
-        <v>46133</v>
+        <v>46160</v>
       </c>
       <c r="G15" s="62">
         <v>1</v>
@@ -19760,7 +19776,7 @@
       </c>
       <c r="F16" s="61">
         <f ca="1">F12+6</f>
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="G16" s="62">
         <v>6</v>
@@ -20241,7 +20257,7 @@
       </c>
       <c r="F18" s="61">
         <f ca="1">F12+6</f>
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="G18" s="62">
         <v>13</v>
@@ -20486,7 +20502,7 @@
       </c>
       <c r="F19" s="61">
         <f ca="1">F18+2</f>
-        <v>46121</v>
+        <v>46148</v>
       </c>
       <c r="G19" s="62">
         <v>9</v>
@@ -20731,7 +20747,7 @@
       </c>
       <c r="F20" s="61">
         <f ca="1">F19+5</f>
-        <v>46126</v>
+        <v>46153</v>
       </c>
       <c r="G20" s="62">
         <v>11</v>
@@ -20974,7 +20990,7 @@
       <c r="E21" s="60"/>
       <c r="F21" s="61">
         <f ca="1">F20+2</f>
-        <v>46128</v>
+        <v>46155</v>
       </c>
       <c r="G21" s="62">
         <v>1</v>
@@ -21215,7 +21231,7 @@
       <c r="E22" s="60"/>
       <c r="F22" s="61">
         <f ca="1">F21+1</f>
-        <v>46129</v>
+        <v>46156</v>
       </c>
       <c r="G22" s="62">
         <v>24</v>
@@ -21694,7 +21710,7 @@
       <c r="E24" s="60"/>
       <c r="F24" s="61">
         <f ca="1">F12+15</f>
-        <v>46128</v>
+        <v>46155</v>
       </c>
       <c r="G24" s="62">
         <v>4</v>
@@ -21937,7 +21953,7 @@
       <c r="E25" s="60"/>
       <c r="F25" s="61">
         <f ca="1">F24+3</f>
-        <v>46131</v>
+        <v>46158</v>
       </c>
       <c r="G25" s="62">
         <v>14</v>
@@ -22180,7 +22196,7 @@
       <c r="E26" s="60"/>
       <c r="F26" s="61">
         <f ca="1">F25+15</f>
-        <v>46146</v>
+        <v>46173</v>
       </c>
       <c r="G26" s="62">
         <v>6</v>
@@ -22423,7 +22439,7 @@
       <c r="E27" s="60"/>
       <c r="F27" s="61">
         <f ca="1">F21+22</f>
-        <v>46150</v>
+        <v>46177</v>
       </c>
       <c r="G27" s="62">
         <v>3</v>
@@ -22666,7 +22682,7 @@
       <c r="E28" s="60"/>
       <c r="F28" s="61">
         <f ca="1">F16</f>
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="G28" s="62">
         <v>19</v>
@@ -23143,7 +23159,7 @@
       <c r="E30" s="60"/>
       <c r="F30" s="61">
         <f ca="1">F27+3</f>
-        <v>46153</v>
+        <v>46180</v>
       </c>
       <c r="G30" s="62">
         <v>15</v>
@@ -23384,7 +23400,7 @@
       <c r="E31" s="60"/>
       <c r="F31" s="61">
         <f ca="1">F30+14</f>
-        <v>46167</v>
+        <v>46194</v>
       </c>
       <c r="G31" s="62">
         <v>5</v>
@@ -23627,7 +23643,7 @@
       <c r="E32" s="60"/>
       <c r="F32" s="61">
         <f ca="1">F31+42</f>
-        <v>46209</v>
+        <v>46236</v>
       </c>
       <c r="G32" s="62">
         <v>1</v>
@@ -24843,15 +24859,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -24868,6 +24875,15 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25147,14 +25163,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -25162,6 +25170,14 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
     <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
     <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>